<commit_message>
SSIS Course - PracticeActivity1
</commit_message>
<xml_diff>
--- a/Sales Data Processing-Project-April2026/project/reports/clean_sales.xlsx
+++ b/Sales Data Processing-Project-April2026/project/reports/clean_sales.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_TeolanGovender_2026\Sales Data Processing-Project-April2026\project\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52349C4C-FC3F-42AF-94CA-794382DEF1C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B766682-5D5B-4235-8A2B-A9AD98EB7393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pivot table" sheetId="3" r:id="rId1"/>
@@ -25,7 +25,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="201" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -197,7 +197,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="&quot;R&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;R&quot;#,##0.00"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -236,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -246,19 +246,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="18">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -278,16 +277,13 @@
       <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;R&quot;#,##0.00"/>
+      <numFmt numFmtId="164" formatCode="&quot;R&quot;#,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;R&quot;#,##0.00"/>
+      <numFmt numFmtId="34" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -299,16 +295,16 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;R&quot;#,##0.00"/>
+      <numFmt numFmtId="164" formatCode="&quot;R&quot;#,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;??_-;_-@_-"/>
+      <numFmt numFmtId="164" formatCode="&quot;R&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -1393,6 +1389,7 @@
     <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
     <c:pageSetup/>
   </c:printSettings>
+  <c:userShapes r:id="rId3"/>
   <c:extLst>
     <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
       <c14:pivotOptions>
@@ -1400,7 +1397,6 @@
         <c14:dropZoneCategories val="1"/>
         <c14:dropZoneData val="1"/>
         <c14:dropZoneSeries val="1"/>
-        <c14:dropZonesVisible val="1"/>
       </c14:pivotOptions>
     </c:ext>
     <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
@@ -1566,6 +1562,9 @@
       <c:pivotFmt>
         <c:idx val="1"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -3965,6 +3964,36 @@
     <c:fmtId val="13"/>
   </c:pivotSource>
   <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:pivotFmts>
       <c:pivotFmt>
@@ -4244,6 +4273,9 @@
       <c:pivotFmt>
         <c:idx val="5"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -9672,6 +9704,90 @@
 <c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
+      <cdr:x>0.03107</cdr:x>
+      <cdr:y>0.2609</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.21633</cdr:x>
+      <cdr:y>0.49575</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A65D0ED0-8907-CE08-B2A1-EE711CC3B724}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="188451" y="879831"/>
+          <a:ext cx="1123736" cy="791967"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="square" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:endParaRPr lang="en-ZA" sz="1100" kern="1200"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.04478</cdr:x>
+      <cdr:y>0.37991</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.09893</cdr:x>
+      <cdr:y>0.55446</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0220A267-421E-E400-4250-0CEB1908C0D5}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="16200000">
+          <a:off x="74917" y="1436350"/>
+          <a:ext cx="588624" cy="278259"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="square" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:r>
+            <a:rPr lang="en-ZA" sz="1100" kern="1200"/>
+            <a:t>Region</a:t>
+          </a:r>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+</c:userShapes>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
       <cdr:x>0.25616</cdr:x>
       <cdr:y>0.89823</cdr:y>
     </cdr:from>
@@ -10445,7 +10561,112 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BE2E50B7-5C0C-4E9D-BBFB-ECDC5A2887F7}" name="Sales by region" cacheId="201" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1BF34DAD-2D29-4EA1-BA89-BA0D733ADA39}" name="Sales Performance for Each Category" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="23">
+  <location ref="A36:B41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="11">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0" sortType="ascending"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item m="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="9"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of quantity" fld="4" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="11">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="3">
+    <chartFormat chart="17" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="18" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="21" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BE2E50B7-5C0C-4E9D-BBFB-ECDC5A2887F7}" name="Sales by region" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -10512,7 +10733,7 @@
   </colItems>
   <dataFields count="2">
     <dataField name="Sum of quantity" fld="4" baseField="6" baseItem="1"/>
-    <dataField name="Sum of revenue" fld="8" baseField="6" baseItem="1" numFmtId="165"/>
+    <dataField name="Sum of revenue" fld="8" baseField="6" baseItem="1" numFmtId="164"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -10526,8 +10747,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DFE920DA-2A0D-40DB-A7F9-1E9016DB83F2}" name="Monthly revenue" cacheId="201" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DFE920DA-2A0D-40DB-A7F9-1E9016DB83F2}" name="Monthly revenue" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A20:B25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -10574,13 +10795,13 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of revenue" fld="8" baseField="9" baseItem="0" numFmtId="165"/>
+    <dataField name="Sum of revenue" fld="8" baseField="9" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="8">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="12">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10602,8 +10823,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B151291E-11D9-4320-8820-3801DB46F4C8}" name="Salesperson performance" cacheId="201" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B151291E-11D9-4320-8820-3801DB46F4C8}" name="Salesperson performance" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
   <location ref="A28:B34" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -10664,13 +10885,13 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of revenue" fld="8" baseField="9" baseItem="0" numFmtId="165"/>
+    <dataField name="Sum of revenue" fld="8" baseField="9" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="10">
+    <format dxfId="15">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="14">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10712,8 +10933,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C6A08E00-819E-42C0-B751-7665F2A20E4A}" name="Product Performance" cacheId="201" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C6A08E00-819E-42C0-B751-7665F2A20E4A}" name="Product Performance" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
   <location ref="A11:C17" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -10796,10 +11017,10 @@
     <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="12">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="16">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10877,113 +11098,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1BF34DAD-2D29-4EA1-BA89-BA0D733ADA39}" name="Sales Performance for Each Category" cacheId="201" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="23">
-  <location ref="A36:B41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="11">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0" sortType="ascending"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item m="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="9"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of quantity" fld="4" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="13">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="3">
-    <chartFormat chart="17" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="18" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="21" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3C8E0B53-DFDF-4BB9-BEF1-9D9488958B24}" name="PivotTable6" cacheId="201" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3C8E0B53-DFDF-4BB9-BEF1-9D9488958B24}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="17">
   <location ref="A8:B13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -11101,13 +11217,13 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of revenue" fld="8" baseField="9" baseItem="0" numFmtId="165"/>
+    <dataField name="Sum of revenue" fld="8" baseField="9" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="15">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="6">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -11141,7 +11257,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3CB6F598-0206-4884-BA11-AF458FEA9674}" name="PivotTable5" cacheId="201" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3CB6F598-0206-4884-BA11-AF458FEA9674}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14">
   <location ref="A1:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -11267,7 +11383,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{21DBC5E3-570C-43D0-83C3-4AB0F012A39E}" name="PivotTable1" cacheId="201" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="42">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{21DBC5E3-570C-43D0-83C3-4AB0F012A39E}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="42">
   <location ref="A25:C31" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -11359,10 +11475,10 @@
     <dataField name="Sum of quantity" fld="4" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="17">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="8">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -11525,7 +11641,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BA627F9E-4A2D-40A8-9E17-92E82BF11E96}" name="PivotTable7" cacheId="201" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BA627F9E-4A2D-40A8-9E17-92E82BF11E96}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
   <location ref="A15:B23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -11664,7 +11780,7 @@
     <dataField name="Sum of quantity" fld="4" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="18">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -12176,7 +12292,7 @@
       <c r="A4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4">
         <v>43</v>
       </c>
       <c r="C4" s="5">
@@ -12187,7 +12303,7 @@
       <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5">
         <v>47</v>
       </c>
       <c r="C5" s="5">
@@ -12198,7 +12314,7 @@
       <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6">
         <v>43</v>
       </c>
       <c r="C6" s="5">
@@ -12209,7 +12325,7 @@
       <c r="A7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7">
         <v>26</v>
       </c>
       <c r="C7" s="5">
@@ -12220,7 +12336,7 @@
       <c r="A8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8">
         <v>159</v>
       </c>
       <c r="C8" s="5">
@@ -12252,7 +12368,7 @@
       <c r="B12" s="6">
         <v>39</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12">
         <v>58500</v>
       </c>
     </row>
@@ -12263,7 +12379,7 @@
       <c r="B13" s="6">
         <v>25</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13">
         <v>75000</v>
       </c>
     </row>
@@ -12274,7 +12390,7 @@
       <c r="B14" s="6">
         <v>15</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14">
         <v>180000</v>
       </c>
     </row>
@@ -12285,7 +12401,7 @@
       <c r="B15" s="6">
         <v>55</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15">
         <v>440000</v>
       </c>
     </row>
@@ -12296,7 +12412,7 @@
       <c r="B16" s="6">
         <v>25</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16">
         <v>150000</v>
       </c>
     </row>
@@ -12307,7 +12423,7 @@
       <c r="B17" s="6">
         <v>159</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17">
         <v>903500</v>
       </c>
     </row>
@@ -12447,7 +12563,7 @@
       <c r="A37" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B37" s="10">
+      <c r="B37">
         <v>21</v>
       </c>
     </row>
@@ -12455,7 +12571,7 @@
       <c r="A38" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38">
         <v>42</v>
       </c>
     </row>
@@ -12463,7 +12579,7 @@
       <c r="A39" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B39" s="10">
+      <c r="B39">
         <v>50</v>
       </c>
     </row>
@@ -12471,7 +12587,7 @@
       <c r="A40" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B40" s="10">
+      <c r="B40">
         <v>46</v>
       </c>
     </row>
@@ -12479,7 +12595,7 @@
       <c r="A41" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B41" s="10">
+      <c r="B41">
         <v>159</v>
       </c>
     </row>
@@ -12504,8 +12620,9 @@
   <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.42578125" customWidth="1"/>
+    <col min="2" max="3" width="15.28515625" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -12520,7 +12637,7 @@
       <c r="A2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2">
         <v>43</v>
       </c>
     </row>
@@ -12528,7 +12645,7 @@
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3">
         <v>47</v>
       </c>
     </row>
@@ -12536,7 +12653,7 @@
       <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4">
         <v>43</v>
       </c>
     </row>
@@ -12544,7 +12661,7 @@
       <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5">
         <v>26</v>
       </c>
     </row>
@@ -12552,7 +12669,7 @@
       <c r="A6" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6">
         <v>159</v>
       </c>
     </row>
@@ -12616,7 +12733,7 @@
       <c r="A16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16">
         <v>95</v>
       </c>
     </row>
@@ -12624,7 +12741,7 @@
       <c r="A17" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17">
         <v>15</v>
       </c>
     </row>
@@ -12632,7 +12749,7 @@
       <c r="A18" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18">
         <v>55</v>
       </c>
     </row>
@@ -12640,7 +12757,7 @@
       <c r="A19" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19">
         <v>25</v>
       </c>
     </row>
@@ -12648,7 +12765,7 @@
       <c r="A20" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20">
         <v>64</v>
       </c>
     </row>
@@ -12656,7 +12773,7 @@
       <c r="A21" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21">
         <v>39</v>
       </c>
     </row>
@@ -12664,7 +12781,7 @@
       <c r="A22" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22">
         <v>25</v>
       </c>
     </row>
@@ -12672,7 +12789,7 @@
       <c r="A23" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="10">
+      <c r="B23">
         <v>159</v>
       </c>
     </row>
@@ -12694,7 +12811,7 @@
       <c r="B26" s="7">
         <v>440000</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26">
         <v>55</v>
       </c>
     </row>
@@ -12705,7 +12822,7 @@
       <c r="B27" s="7">
         <v>180000</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27">
         <v>15</v>
       </c>
     </row>
@@ -12716,7 +12833,7 @@
       <c r="B28" s="7">
         <v>150000</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C28">
         <v>25</v>
       </c>
     </row>
@@ -12727,7 +12844,7 @@
       <c r="B29" s="7">
         <v>75000</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C29">
         <v>25</v>
       </c>
     </row>
@@ -12738,7 +12855,7 @@
       <c r="B30" s="7">
         <v>58500</v>
       </c>
-      <c r="C30" s="10">
+      <c r="C30">
         <v>39</v>
       </c>
     </row>
@@ -12749,7 +12866,7 @@
       <c r="B31" s="7">
         <v>903500</v>
       </c>
-      <c r="C31" s="10">
+      <c r="C31">
         <v>159</v>
       </c>
     </row>
@@ -12827,10 +12944,10 @@
       <c r="B2" s="1">
         <v>45296</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" t="s">
         <v>11</v>
       </c>
       <c r="E2">
@@ -12839,16 +12956,16 @@
       <c r="F2">
         <v>12000</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" t="s">
         <v>13</v>
       </c>
       <c r="I2">
         <v>24000</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="J2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -12859,10 +12976,10 @@
       <c r="B3" s="1">
         <v>45298</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" t="s">
         <v>11</v>
       </c>
       <c r="E3">
@@ -12871,16 +12988,16 @@
       <c r="F3">
         <v>8000</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" t="s">
         <v>17</v>
       </c>
       <c r="I3">
         <v>40000</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J3" t="s">
         <v>14</v>
       </c>
     </row>
@@ -12891,10 +13008,10 @@
       <c r="B4" s="1">
         <v>45301</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="E4">
@@ -12903,16 +13020,16 @@
       <c r="F4">
         <v>6000</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" t="s">
         <v>20</v>
       </c>
       <c r="I4">
         <v>18000</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" t="s">
         <v>14</v>
       </c>
     </row>
@@ -12923,10 +13040,10 @@
       <c r="B5" s="1">
         <v>45311</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" t="s">
         <v>22</v>
       </c>
       <c r="E5">
@@ -12935,16 +13052,16 @@
       <c r="F5">
         <v>3000</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" t="s">
         <v>13</v>
       </c>
       <c r="I5">
         <v>6000</v>
       </c>
-      <c r="J5" s="10" t="s">
+      <c r="J5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -12955,10 +13072,10 @@
       <c r="B6" s="1">
         <v>45313</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6">
@@ -12967,16 +13084,16 @@
       <c r="F6">
         <v>12000</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" t="s">
         <v>17</v>
       </c>
       <c r="I6">
         <v>12000</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="J6" t="s">
         <v>14</v>
       </c>
     </row>
@@ -12987,10 +13104,10 @@
       <c r="B7" s="1">
         <v>45316</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7">
@@ -12999,16 +13116,16 @@
       <c r="F7">
         <v>8000</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" t="s">
         <v>20</v>
       </c>
       <c r="I7">
         <v>48000</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="J7" t="s">
         <v>14</v>
       </c>
     </row>
@@ -13019,10 +13136,10 @@
       <c r="B8" s="1">
         <v>45319</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" t="s">
         <v>11</v>
       </c>
       <c r="E8">
@@ -13031,16 +13148,16 @@
       <c r="F8">
         <v>6000</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" t="s">
         <v>24</v>
       </c>
       <c r="I8">
         <v>12000</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="J8" t="s">
         <v>14</v>
       </c>
     </row>
@@ -13051,10 +13168,10 @@
       <c r="B9" s="1">
         <v>45323</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" t="s">
         <v>22</v>
       </c>
       <c r="E9">
@@ -13063,16 +13180,16 @@
       <c r="F9">
         <v>1500</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" t="s">
         <v>13</v>
       </c>
       <c r="I9">
         <v>7500</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13083,10 +13200,10 @@
       <c r="B10" s="1">
         <v>45325</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" t="s">
         <v>22</v>
       </c>
       <c r="E10">
@@ -13095,16 +13212,16 @@
       <c r="F10">
         <v>3000</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" t="s">
         <v>38</v>
       </c>
       <c r="I10">
         <v>9000</v>
       </c>
-      <c r="J10" s="10" t="s">
+      <c r="J10" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13115,10 +13232,10 @@
       <c r="B11" s="1">
         <v>45327</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11">
@@ -13127,16 +13244,16 @@
       <c r="F11">
         <v>12000</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" t="s">
         <v>19</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" t="s">
         <v>20</v>
       </c>
       <c r="I11">
         <v>24000</v>
       </c>
-      <c r="J11" s="10" t="s">
+      <c r="J11" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13147,10 +13264,10 @@
       <c r="B12" s="1">
         <v>45329</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" t="s">
         <v>11</v>
       </c>
       <c r="E12">
@@ -13159,16 +13276,16 @@
       <c r="F12">
         <v>8000</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" t="s">
         <v>24</v>
       </c>
       <c r="I12">
         <v>32000</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="J12" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13179,10 +13296,10 @@
       <c r="B13" s="1">
         <v>45332</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" t="s">
         <v>11</v>
       </c>
       <c r="E13">
@@ -13191,16 +13308,16 @@
       <c r="F13">
         <v>6000</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="G13" t="s">
         <v>12</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" t="s">
         <v>13</v>
       </c>
       <c r="I13">
         <v>18000</v>
       </c>
-      <c r="J13" s="10" t="s">
+      <c r="J13" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13211,10 +13328,10 @@
       <c r="B14" s="1">
         <v>45334</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" t="s">
         <v>22</v>
       </c>
       <c r="E14">
@@ -13223,16 +13340,16 @@
       <c r="F14">
         <v>1500</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="G14" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H14" t="s">
         <v>17</v>
       </c>
       <c r="I14">
         <v>9000</v>
       </c>
-      <c r="J14" s="10" t="s">
+      <c r="J14" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13243,10 +13360,10 @@
       <c r="B15" s="1">
         <v>45337</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" t="s">
         <v>22</v>
       </c>
       <c r="E15">
@@ -13255,16 +13372,16 @@
       <c r="F15">
         <v>3000</v>
       </c>
-      <c r="G15" s="10" t="s">
+      <c r="G15" t="s">
         <v>19</v>
       </c>
-      <c r="H15" s="10" t="s">
+      <c r="H15" t="s">
         <v>20</v>
       </c>
       <c r="I15">
         <v>6000</v>
       </c>
-      <c r="J15" s="10" t="s">
+      <c r="J15" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13275,10 +13392,10 @@
       <c r="B16" s="1">
         <v>45340</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" t="s">
         <v>11</v>
       </c>
       <c r="E16">
@@ -13287,16 +13404,16 @@
       <c r="F16">
         <v>12000</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="G16" t="s">
         <v>23</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="H16" t="s">
         <v>24</v>
       </c>
       <c r="I16">
         <v>12000</v>
       </c>
-      <c r="J16" s="10" t="s">
+      <c r="J16" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13307,10 +13424,10 @@
       <c r="B17" s="1">
         <v>45342</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" t="s">
         <v>15</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" t="s">
         <v>11</v>
       </c>
       <c r="E17">
@@ -13319,16 +13436,16 @@
       <c r="F17">
         <v>8000</v>
       </c>
-      <c r="G17" s="10" t="s">
+      <c r="G17" t="s">
         <v>12</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" t="s">
         <v>13</v>
       </c>
       <c r="I17">
         <v>56000</v>
       </c>
-      <c r="J17" s="10" t="s">
+      <c r="J17" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13339,10 +13456,10 @@
       <c r="B18" s="1">
         <v>45344</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" t="s">
         <v>18</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" t="s">
         <v>11</v>
       </c>
       <c r="E18">
@@ -13351,16 +13468,16 @@
       <c r="F18">
         <v>6000</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="G18" t="s">
         <v>16</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" t="s">
         <v>17</v>
       </c>
       <c r="I18">
         <v>12000</v>
       </c>
-      <c r="J18" s="10" t="s">
+      <c r="J18" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13371,10 +13488,10 @@
       <c r="B19" s="1">
         <v>45347</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" t="s">
         <v>22</v>
       </c>
       <c r="E19">
@@ -13383,16 +13500,16 @@
       <c r="F19">
         <v>1500</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="G19" t="s">
         <v>19</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="H19" t="s">
         <v>20</v>
       </c>
       <c r="I19">
         <v>6000</v>
       </c>
-      <c r="J19" s="10" t="s">
+      <c r="J19" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13403,10 +13520,10 @@
       <c r="B20" s="1">
         <v>45350</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" t="s">
         <v>22</v>
       </c>
       <c r="E20">
@@ -13415,16 +13532,16 @@
       <c r="F20">
         <v>3000</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="G20" t="s">
         <v>23</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="H20" t="s">
         <v>24</v>
       </c>
       <c r="I20">
         <v>9000</v>
       </c>
-      <c r="J20" s="10" t="s">
+      <c r="J20" t="s">
         <v>26</v>
       </c>
     </row>
@@ -13435,10 +13552,10 @@
       <c r="B21" s="1">
         <v>45353</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" t="s">
         <v>11</v>
       </c>
       <c r="E21">
@@ -13447,16 +13564,16 @@
       <c r="F21">
         <v>12000</v>
       </c>
-      <c r="G21" s="10" t="s">
+      <c r="G21" t="s">
         <v>12</v>
       </c>
-      <c r="H21" s="10" t="s">
+      <c r="H21" t="s">
         <v>13</v>
       </c>
       <c r="I21">
         <v>24000</v>
       </c>
-      <c r="J21" s="10" t="s">
+      <c r="J21" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13467,10 +13584,10 @@
       <c r="B22" s="1">
         <v>45355</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" t="s">
         <v>11</v>
       </c>
       <c r="E22">
@@ -13479,16 +13596,16 @@
       <c r="F22">
         <v>8000</v>
       </c>
-      <c r="G22" s="10" t="s">
+      <c r="G22" t="s">
         <v>16</v>
       </c>
-      <c r="H22" s="10" t="s">
+      <c r="H22" t="s">
         <v>17</v>
       </c>
       <c r="I22">
         <v>40000</v>
       </c>
-      <c r="J22" s="10" t="s">
+      <c r="J22" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13499,10 +13616,10 @@
       <c r="B23" s="1">
         <v>45357</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" t="s">
         <v>18</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" t="s">
         <v>11</v>
       </c>
       <c r="E23">
@@ -13511,16 +13628,16 @@
       <c r="F23">
         <v>6000</v>
       </c>
-      <c r="G23" s="10" t="s">
+      <c r="G23" t="s">
         <v>19</v>
       </c>
-      <c r="H23" s="10" t="s">
+      <c r="H23" t="s">
         <v>20</v>
       </c>
       <c r="I23">
         <v>18000</v>
       </c>
-      <c r="J23" s="10" t="s">
+      <c r="J23" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13531,10 +13648,10 @@
       <c r="B24" s="1">
         <v>45359</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" t="s">
         <v>21</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" t="s">
         <v>22</v>
       </c>
       <c r="E24">
@@ -13543,16 +13660,16 @@
       <c r="F24">
         <v>1500</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="G24" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="10" t="s">
+      <c r="H24" t="s">
         <v>24</v>
       </c>
       <c r="I24">
         <v>6000</v>
       </c>
-      <c r="J24" s="10" t="s">
+      <c r="J24" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13563,10 +13680,10 @@
       <c r="B25" s="1">
         <v>45361</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" t="s">
         <v>22</v>
       </c>
       <c r="E25">
@@ -13575,16 +13692,16 @@
       <c r="F25">
         <v>3000</v>
       </c>
-      <c r="G25" s="10" t="s">
+      <c r="G25" t="s">
         <v>12</v>
       </c>
-      <c r="H25" s="10" t="s">
+      <c r="H25" t="s">
         <v>13</v>
       </c>
       <c r="I25">
         <v>6000</v>
       </c>
-      <c r="J25" s="10" t="s">
+      <c r="J25" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13595,10 +13712,10 @@
       <c r="B26" s="1">
         <v>45363</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" t="s">
         <v>10</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26">
@@ -13607,16 +13724,16 @@
       <c r="F26">
         <v>12000</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="G26" t="s">
         <v>16</v>
       </c>
-      <c r="H26" s="10" t="s">
+      <c r="H26" t="s">
         <v>17</v>
       </c>
       <c r="I26">
         <v>12000</v>
       </c>
-      <c r="J26" s="10" t="s">
+      <c r="J26" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13627,10 +13744,10 @@
       <c r="B27" s="1">
         <v>45365</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" t="s">
         <v>15</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27">
@@ -13639,16 +13756,16 @@
       <c r="F27">
         <v>8000</v>
       </c>
-      <c r="G27" s="10" t="s">
+      <c r="G27" t="s">
         <v>19</v>
       </c>
-      <c r="H27" s="10" t="s">
+      <c r="H27" t="s">
         <v>20</v>
       </c>
       <c r="I27">
         <v>48000</v>
       </c>
-      <c r="J27" s="10" t="s">
+      <c r="J27" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13659,10 +13776,10 @@
       <c r="B28" s="1">
         <v>45367</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" t="s">
         <v>18</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28">
@@ -13671,16 +13788,16 @@
       <c r="F28">
         <v>6000</v>
       </c>
-      <c r="G28" s="10" t="s">
+      <c r="G28" t="s">
         <v>23</v>
       </c>
-      <c r="H28" s="10" t="s">
+      <c r="H28" t="s">
         <v>24</v>
       </c>
       <c r="I28">
         <v>12000</v>
       </c>
-      <c r="J28" s="10" t="s">
+      <c r="J28" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13691,10 +13808,10 @@
       <c r="B29" s="1">
         <v>45369</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" t="s">
         <v>21</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" t="s">
         <v>22</v>
       </c>
       <c r="E29">
@@ -13703,16 +13820,16 @@
       <c r="F29">
         <v>1500</v>
       </c>
-      <c r="G29" s="10" t="s">
+      <c r="G29" t="s">
         <v>12</v>
       </c>
-      <c r="H29" s="10" t="s">
+      <c r="H29" t="s">
         <v>13</v>
       </c>
       <c r="I29">
         <v>7500</v>
       </c>
-      <c r="J29" s="10" t="s">
+      <c r="J29" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13723,10 +13840,10 @@
       <c r="B30" s="1">
         <v>45371</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" t="s">
         <v>25</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" t="s">
         <v>22</v>
       </c>
       <c r="E30">
@@ -13735,16 +13852,16 @@
       <c r="F30">
         <v>3000</v>
       </c>
-      <c r="G30" s="10" t="s">
+      <c r="G30" t="s">
         <v>16</v>
       </c>
-      <c r="H30" s="10" t="s">
+      <c r="H30" t="s">
         <v>17</v>
       </c>
       <c r="I30">
         <v>9000</v>
       </c>
-      <c r="J30" s="10" t="s">
+      <c r="J30" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13755,10 +13872,10 @@
       <c r="B31" s="1">
         <v>45373</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" t="s">
         <v>10</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="D31" t="s">
         <v>11</v>
       </c>
       <c r="E31">
@@ -13767,16 +13884,16 @@
       <c r="F31">
         <v>12000</v>
       </c>
-      <c r="G31" s="10" t="s">
+      <c r="G31" t="s">
         <v>19</v>
       </c>
-      <c r="H31" s="10" t="s">
+      <c r="H31" t="s">
         <v>20</v>
       </c>
       <c r="I31">
         <v>24000</v>
       </c>
-      <c r="J31" s="10" t="s">
+      <c r="J31" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13787,10 +13904,10 @@
       <c r="B32" s="1">
         <v>45375</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" t="s">
         <v>15</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32">
@@ -13799,16 +13916,16 @@
       <c r="F32">
         <v>8000</v>
       </c>
-      <c r="G32" s="10" t="s">
+      <c r="G32" t="s">
         <v>23</v>
       </c>
-      <c r="H32" s="10" t="s">
+      <c r="H32" t="s">
         <v>24</v>
       </c>
       <c r="I32">
         <v>32000</v>
       </c>
-      <c r="J32" s="10" t="s">
+      <c r="J32" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13819,10 +13936,10 @@
       <c r="B33" s="1">
         <v>45377</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" t="s">
         <v>18</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D33" t="s">
         <v>11</v>
       </c>
       <c r="E33">
@@ -13831,16 +13948,16 @@
       <c r="F33">
         <v>6000</v>
       </c>
-      <c r="G33" s="10" t="s">
+      <c r="G33" t="s">
         <v>12</v>
       </c>
-      <c r="H33" s="10" t="s">
+      <c r="H33" t="s">
         <v>13</v>
       </c>
       <c r="I33">
         <v>18000</v>
       </c>
-      <c r="J33" s="10" t="s">
+      <c r="J33" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13851,10 +13968,10 @@
       <c r="B34" s="1">
         <v>45379</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C34" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="D34" t="s">
         <v>22</v>
       </c>
       <c r="E34">
@@ -13863,16 +13980,16 @@
       <c r="F34">
         <v>1500</v>
       </c>
-      <c r="G34" s="10" t="s">
+      <c r="G34" t="s">
         <v>16</v>
       </c>
-      <c r="H34" s="10" t="s">
+      <c r="H34" t="s">
         <v>17</v>
       </c>
       <c r="I34">
         <v>9000</v>
       </c>
-      <c r="J34" s="10" t="s">
+      <c r="J34" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13883,10 +14000,10 @@
       <c r="B35" s="1">
         <v>45381</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="C35" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" t="s">
         <v>22</v>
       </c>
       <c r="E35">
@@ -13895,16 +14012,16 @@
       <c r="F35">
         <v>3000</v>
       </c>
-      <c r="G35" s="10" t="s">
+      <c r="G35" t="s">
         <v>19</v>
       </c>
-      <c r="H35" s="10" t="s">
+      <c r="H35" t="s">
         <v>20</v>
       </c>
       <c r="I35">
         <v>6000</v>
       </c>
-      <c r="J35" s="10" t="s">
+      <c r="J35" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13915,10 +14032,10 @@
       <c r="B36" s="1">
         <v>45384</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="C36" t="s">
         <v>10</v>
       </c>
-      <c r="D36" s="10" t="s">
+      <c r="D36" t="s">
         <v>11</v>
       </c>
       <c r="E36">
@@ -13927,16 +14044,16 @@
       <c r="F36">
         <v>12000</v>
       </c>
-      <c r="G36" s="10" t="s">
+      <c r="G36" t="s">
         <v>23</v>
       </c>
-      <c r="H36" s="10" t="s">
+      <c r="H36" t="s">
         <v>24</v>
       </c>
       <c r="I36">
         <v>12000</v>
       </c>
-      <c r="J36" s="10" t="s">
+      <c r="J36" t="s">
         <v>28</v>
       </c>
     </row>
@@ -13947,10 +14064,10 @@
       <c r="B37" s="1">
         <v>45386</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="C37" t="s">
         <v>15</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D37" t="s">
         <v>11</v>
       </c>
       <c r="E37">
@@ -13959,16 +14076,16 @@
       <c r="F37">
         <v>8000</v>
       </c>
-      <c r="G37" s="10" t="s">
+      <c r="G37" t="s">
         <v>12</v>
       </c>
-      <c r="H37" s="10" t="s">
+      <c r="H37" t="s">
         <v>13</v>
       </c>
       <c r="I37">
         <v>56000</v>
       </c>
-      <c r="J37" s="10" t="s">
+      <c r="J37" t="s">
         <v>28</v>
       </c>
     </row>
@@ -13979,10 +14096,10 @@
       <c r="B38" s="1">
         <v>45388</v>
       </c>
-      <c r="C38" s="10" t="s">
+      <c r="C38" t="s">
         <v>18</v>
       </c>
-      <c r="D38" s="10" t="s">
+      <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="E38">
@@ -13991,16 +14108,16 @@
       <c r="F38">
         <v>6000</v>
       </c>
-      <c r="G38" s="10" t="s">
+      <c r="G38" t="s">
         <v>16</v>
       </c>
-      <c r="H38" s="10" t="s">
+      <c r="H38" t="s">
         <v>17</v>
       </c>
       <c r="I38">
         <v>12000</v>
       </c>
-      <c r="J38" s="10" t="s">
+      <c r="J38" t="s">
         <v>28</v>
       </c>
     </row>
@@ -14011,10 +14128,10 @@
       <c r="B39" s="1">
         <v>45390</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" t="s">
         <v>21</v>
       </c>
-      <c r="D39" s="10" t="s">
+      <c r="D39" t="s">
         <v>22</v>
       </c>
       <c r="E39">
@@ -14023,16 +14140,16 @@
       <c r="F39">
         <v>1500</v>
       </c>
-      <c r="G39" s="10" t="s">
+      <c r="G39" t="s">
         <v>19</v>
       </c>
-      <c r="H39" s="10" t="s">
+      <c r="H39" t="s">
         <v>20</v>
       </c>
       <c r="I39">
         <v>6000</v>
       </c>
-      <c r="J39" s="10" t="s">
+      <c r="J39" t="s">
         <v>28</v>
       </c>
     </row>
@@ -14043,10 +14160,10 @@
       <c r="B40" s="1">
         <v>45392</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="10" t="s">
+      <c r="D40" t="s">
         <v>22</v>
       </c>
       <c r="E40">
@@ -14055,16 +14172,16 @@
       <c r="F40">
         <v>3000</v>
       </c>
-      <c r="G40" s="10" t="s">
+      <c r="G40" t="s">
         <v>23</v>
       </c>
-      <c r="H40" s="10" t="s">
+      <c r="H40" t="s">
         <v>24</v>
       </c>
       <c r="I40">
         <v>9000</v>
       </c>
-      <c r="J40" s="10" t="s">
+      <c r="J40" t="s">
         <v>28</v>
       </c>
     </row>
@@ -14075,10 +14192,10 @@
       <c r="B41" s="1">
         <v>45394</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" t="s">
         <v>10</v>
       </c>
-      <c r="D41" s="10" t="s">
+      <c r="D41" t="s">
         <v>11</v>
       </c>
       <c r="E41">
@@ -14087,16 +14204,16 @@
       <c r="F41">
         <v>12000</v>
       </c>
-      <c r="G41" s="10" t="s">
+      <c r="G41" t="s">
         <v>12</v>
       </c>
-      <c r="H41" s="10" t="s">
+      <c r="H41" t="s">
         <v>13</v>
       </c>
       <c r="I41">
         <v>24000</v>
       </c>
-      <c r="J41" s="10" t="s">
+      <c r="J41" t="s">
         <v>28</v>
       </c>
     </row>
@@ -14107,10 +14224,10 @@
       <c r="B42" s="1">
         <v>45396</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" t="s">
         <v>15</v>
       </c>
-      <c r="D42" s="10" t="s">
+      <c r="D42" t="s">
         <v>11</v>
       </c>
       <c r="E42">
@@ -14119,16 +14236,16 @@
       <c r="F42">
         <v>8000</v>
       </c>
-      <c r="G42" s="10" t="s">
+      <c r="G42" t="s">
         <v>16</v>
       </c>
-      <c r="H42" s="10" t="s">
+      <c r="H42" t="s">
         <v>17</v>
       </c>
       <c r="I42">
         <v>40000</v>
       </c>
-      <c r="J42" s="10" t="s">
+      <c r="J42" t="s">
         <v>28</v>
       </c>
     </row>
@@ -14139,10 +14256,10 @@
       <c r="B43" s="1">
         <v>45398</v>
       </c>
-      <c r="C43" s="10" t="s">
+      <c r="C43" t="s">
         <v>18</v>
       </c>
-      <c r="D43" s="10" t="s">
+      <c r="D43" t="s">
         <v>11</v>
       </c>
       <c r="E43">
@@ -14151,16 +14268,16 @@
       <c r="F43">
         <v>6000</v>
       </c>
-      <c r="G43" s="10" t="s">
+      <c r="G43" t="s">
         <v>19</v>
       </c>
-      <c r="H43" s="10" t="s">
+      <c r="H43" t="s">
         <v>20</v>
       </c>
       <c r="I43">
         <v>18000</v>
       </c>
-      <c r="J43" s="10" t="s">
+      <c r="J43" t="s">
         <v>28</v>
       </c>
     </row>
@@ -14171,10 +14288,10 @@
       <c r="B44" s="1">
         <v>45402</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="C44" t="s">
         <v>25</v>
       </c>
-      <c r="D44" s="10" t="s">
+      <c r="D44" t="s">
         <v>22</v>
       </c>
       <c r="E44">
@@ -14183,16 +14300,16 @@
       <c r="F44">
         <v>3000</v>
       </c>
-      <c r="G44" s="10" t="s">
+      <c r="G44" t="s">
         <v>12</v>
       </c>
-      <c r="H44" s="10" t="s">
+      <c r="H44" t="s">
         <v>13</v>
       </c>
       <c r="I44">
         <v>6000</v>
       </c>
-      <c r="J44" s="10" t="s">
+      <c r="J44" t="s">
         <v>28</v>
       </c>
     </row>
@@ -14203,10 +14320,10 @@
       <c r="B45" s="1">
         <v>45404</v>
       </c>
-      <c r="C45" s="10" t="s">
+      <c r="C45" t="s">
         <v>10</v>
       </c>
-      <c r="D45" s="10" t="s">
+      <c r="D45" t="s">
         <v>11</v>
       </c>
       <c r="E45">
@@ -14215,16 +14332,16 @@
       <c r="F45">
         <v>12000</v>
       </c>
-      <c r="G45" s="10" t="s">
+      <c r="G45" t="s">
         <v>16</v>
       </c>
-      <c r="H45" s="10" t="s">
+      <c r="H45" t="s">
         <v>38</v>
       </c>
       <c r="I45">
         <v>12000</v>
       </c>
-      <c r="J45" s="10" t="s">
+      <c r="J45" t="s">
         <v>28</v>
       </c>
     </row>
@@ -14235,10 +14352,10 @@
       <c r="B46" s="1">
         <v>45406</v>
       </c>
-      <c r="C46" s="10" t="s">
+      <c r="C46" t="s">
         <v>15</v>
       </c>
-      <c r="D46" s="10" t="s">
+      <c r="D46" t="s">
         <v>11</v>
       </c>
       <c r="E46">
@@ -14247,16 +14364,16 @@
       <c r="F46">
         <v>8000</v>
       </c>
-      <c r="G46" s="10" t="s">
+      <c r="G46" t="s">
         <v>19</v>
       </c>
-      <c r="H46" s="10" t="s">
+      <c r="H46" t="s">
         <v>20</v>
       </c>
       <c r="I46">
         <v>48000</v>
       </c>
-      <c r="J46" s="10" t="s">
+      <c r="J46" t="s">
         <v>28</v>
       </c>
     </row>
@@ -14267,10 +14384,10 @@
       <c r="B47" s="1">
         <v>45408</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="C47" t="s">
         <v>18</v>
       </c>
-      <c r="D47" s="10" t="s">
+      <c r="D47" t="s">
         <v>11</v>
       </c>
       <c r="E47">
@@ -14279,16 +14396,16 @@
       <c r="F47">
         <v>6000</v>
       </c>
-      <c r="G47" s="10" t="s">
+      <c r="G47" t="s">
         <v>23</v>
       </c>
-      <c r="H47" s="10" t="s">
+      <c r="H47" t="s">
         <v>24</v>
       </c>
       <c r="I47">
         <v>12000</v>
       </c>
-      <c r="J47" s="10" t="s">
+      <c r="J47" t="s">
         <v>28</v>
       </c>
     </row>
@@ -14299,10 +14416,10 @@
       <c r="B48" s="1">
         <v>45410</v>
       </c>
-      <c r="C48" s="10" t="s">
+      <c r="C48" t="s">
         <v>21</v>
       </c>
-      <c r="D48" s="10" t="s">
+      <c r="D48" t="s">
         <v>22</v>
       </c>
       <c r="E48">
@@ -14311,16 +14428,16 @@
       <c r="F48">
         <v>1500</v>
       </c>
-      <c r="G48" s="10" t="s">
+      <c r="G48" t="s">
         <v>12</v>
       </c>
-      <c r="H48" s="10" t="s">
+      <c r="H48" t="s">
         <v>13</v>
       </c>
       <c r="I48">
         <v>7500</v>
       </c>
-      <c r="J48" s="10" t="s">
+      <c r="J48" t="s">
         <v>28</v>
       </c>
     </row>
@@ -14331,10 +14448,10 @@
       <c r="B49" s="1">
         <v>45412</v>
       </c>
-      <c r="C49" s="10" t="s">
+      <c r="C49" t="s">
         <v>25</v>
       </c>
-      <c r="D49" s="10" t="s">
+      <c r="D49" t="s">
         <v>22</v>
       </c>
       <c r="E49">
@@ -14343,16 +14460,16 @@
       <c r="F49">
         <v>3000</v>
       </c>
-      <c r="G49" s="10" t="s">
+      <c r="G49" t="s">
         <v>16</v>
       </c>
-      <c r="H49" s="10" t="s">
+      <c r="H49" t="s">
         <v>17</v>
       </c>
       <c r="I49">
         <v>9000</v>
       </c>
-      <c r="J49" s="10" t="s">
+      <c r="J49" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
T-SQL Course - Completed Session 2
</commit_message>
<xml_diff>
--- a/Sales Data Processing-Project-April2026/project/reports/clean_sales.xlsx
+++ b/Sales Data Processing-Project-April2026/project/reports/clean_sales.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_TeolanGovender_2026\Sales Data Processing-Project-April2026\project\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B766682-5D5B-4235-8A2B-A9AD98EB7393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A323131C-2BF4-4291-B61A-DBCD17C2F6F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pivot table" sheetId="3" r:id="rId1"/>
@@ -283,7 +283,10 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;??_-;_-@_-"/>
+      <numFmt numFmtId="164" formatCode="&quot;R&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -301,10 +304,7 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;R&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <numFmt numFmtId="34" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -3965,6 +3965,36 @@
   </c:pivotSource>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.52539727979637374"/>
+          <c:y val="0.1052915263154848"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -8995,7 +9025,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>27</xdr:col>
-      <xdr:colOff>102742</xdr:colOff>
+      <xdr:colOff>102741</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>96167</xdr:rowOff>
     </xdr:to>
@@ -9276,7 +9306,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>34</xdr:col>
-      <xdr:colOff>4857</xdr:colOff>
+      <xdr:colOff>4858</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>149678</xdr:rowOff>
     </xdr:to>
@@ -9788,12 +9818,12 @@
 <c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
-      <cdr:x>0.25616</cdr:x>
-      <cdr:y>0.89823</cdr:y>
+      <cdr:x>0.27995</cdr:x>
+      <cdr:y>0.07563</cdr:y>
     </cdr:from>
     <cdr:to>
-      <cdr:x>0.72906</cdr:x>
-      <cdr:y>0.99115</cdr:y>
+      <cdr:x>0.75285</cdr:x>
+      <cdr:y>0.16855</cdr:y>
     </cdr:to>
     <cdr:sp macro="" textlink="">
       <cdr:nvSpPr>
@@ -9808,8 +9838,8 @@
       </cdr:nvSpPr>
       <cdr:spPr>
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="1415142" y="2762251"/>
-          <a:ext cx="2612572" cy="285750"/>
+          <a:off x="1259544" y="235175"/>
+          <a:ext cx="2127682" cy="288931"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <a:avLst/>
@@ -10561,111 +10591,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1BF34DAD-2D29-4EA1-BA89-BA0D733ADA39}" name="Sales Performance for Each Category" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="23">
-  <location ref="A36:B41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="11">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0" sortType="ascending"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item m="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="9"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of quantity" fld="4" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="11">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="3">
-    <chartFormat chart="17" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="18" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="21" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BE2E50B7-5C0C-4E9D-BBFB-ECDC5A2887F7}" name="Sales by region" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
@@ -10747,7 +10672,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DFE920DA-2A0D-40DB-A7F9-1E9016DB83F2}" name="Monthly revenue" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A20:B25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
@@ -10798,10 +10723,10 @@
     <dataField name="Sum of revenue" fld="8" baseField="9" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="13">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="6">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10823,7 +10748,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B151291E-11D9-4320-8820-3801DB46F4C8}" name="Salesperson performance" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
   <location ref="A28:B34" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
@@ -10888,10 +10813,10 @@
     <dataField name="Sum of revenue" fld="8" baseField="9" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="15">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="8">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10933,7 +10858,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C6A08E00-819E-42C0-B751-7665F2A20E4A}" name="Product Performance" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
   <location ref="A11:C17" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
@@ -11017,10 +10942,10 @@
     <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="17">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="10">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -11098,8 +11023,113 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1BF34DAD-2D29-4EA1-BA89-BA0D733ADA39}" name="Sales Performance for Each Category" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="23">
+  <location ref="A36:B41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="11">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0" sortType="ascending"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item m="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="9"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of quantity" fld="4" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="12">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="3">
+    <chartFormat chart="17" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="18" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="21" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3C8E0B53-DFDF-4BB9-BEF1-9D9488958B24}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="17">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3C8E0B53-DFDF-4BB9-BEF1-9D9488958B24}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="18">
   <location ref="A8:B13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -11220,10 +11250,10 @@
     <dataField name="Sum of revenue" fld="8" baseField="9" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="7">
+    <format dxfId="14">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="13">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -11257,7 +11287,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3CB6F598-0206-4884-BA11-AF458FEA9674}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3CB6F598-0206-4884-BA11-AF458FEA9674}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
   <location ref="A1:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -11383,7 +11413,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{21DBC5E3-570C-43D0-83C3-4AB0F012A39E}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="42">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{21DBC5E3-570C-43D0-83C3-4AB0F012A39E}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="43">
   <location ref="A25:C31" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -11475,10 +11505,10 @@
     <dataField name="Sum of quantity" fld="4" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="9">
+    <format dxfId="16">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="8">
+    <format dxfId="15">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -11780,7 +11810,7 @@
     <dataField name="Sum of quantity" fld="4" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="10">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -12620,8 +12650,9 @@
   <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" customWidth="1"/>
-    <col min="2" max="3" width="15.28515625" customWidth="1"/>
+    <col min="1" max="1" width="13.42578125" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" customWidth="1"/>
     <col min="4" max="4" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>